<commit_message>
[00 26 07 26 01]更新： 1.新增readme.md文件
</commit_message>
<xml_diff>
--- a/02_DataProcess/01_Ashares/01_DaliyUpdate/活跃市值多空区间.xlsx
+++ b/02_DataProcess/01_Ashares/01_DaliyUpdate/活跃市值多空区间.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Quant\01_SwProj\04_VectorBT\02_Lima\Lima_Gen1\02_DataProcess\01_Ashares\01_DaliyUpdate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AF8B2FB-487F-4B86-98ED-6F2659606B11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{246D6B47-03E5-465F-A8DA-EE22D0FAD9B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4290" yWindow="4290" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>Start</t>
   </si>
@@ -29,6 +29,10 @@
   </si>
   <si>
     <t>Long</t>
+  </si>
+  <si>
+    <t>now</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -359,7 +363,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C78"/>
+  <dimension ref="A1:C79"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="11.125" style="1" bestFit="1" customWidth="1"/>
@@ -1224,6 +1228,17 @@
         <v>1</v>
       </c>
     </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A79" s="2">
+        <v>46202</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C79" s="1">
+        <v>-1</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>